<commit_message>
dmos file with compensated scores
</commit_message>
<xml_diff>
--- a/dmos.xlsx
+++ b/dmos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Desktop/PhD/paper6/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE150D87-C773-704A-B0FF-92DE81FED985}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8514B82A-67A2-754C-88F2-233137F79F08}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16000" firstSheet="9" activeTab="18" xr2:uid="{C66D1F0E-21EA-F246-93F3-1139907156B8}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="14040" firstSheet="10" activeTab="18" xr2:uid="{C66D1F0E-21EA-F246-93F3-1139907156B8}"/>
   </bookViews>
   <sheets>
     <sheet name="participant1" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,9 @@
     <sheet name="participant16" sheetId="16" r:id="rId16"/>
     <sheet name="participant17" sheetId="17" r:id="rId17"/>
     <sheet name="participant18" sheetId="18" r:id="rId18"/>
-    <sheet name="Sheet19" sheetId="19" r:id="rId19"/>
+    <sheet name="dmos" sheetId="19" r:id="rId19"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12161" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12162" uniqueCount="339">
   <si>
     <t>sequenceA</t>
   </si>
@@ -1058,6 +1058,9 @@
   <si>
     <t>DMOS</t>
   </si>
+  <si>
+    <t>DMOS (compensated)</t>
+  </si>
 </sst>
 </file>
 
@@ -46317,7 +46320,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC10506B-31AB-EE4E-8566-3E3C20E43CD6}">
-  <dimension ref="A1:E319"/>
+  <dimension ref="A1:F319"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35" bestFit="1" customWidth="1"/>
@@ -46325,7 +46328,7 @@
     <col min="3" max="3" width="49" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -46341,8 +46344,11 @@
       <c r="E1" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F1" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -46359,7 +46365,7 @@
         <v>5.0341111111111099</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -46376,7 +46382,7 @@
         <v>5.3753555555555561</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
@@ -46393,7 +46399,7 @@
         <v>5.2287555555555567</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
@@ -46410,7 +46416,7 @@
         <v>4.5579999999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>10</v>
       </c>
@@ -46427,7 +46433,7 @@
         <v>5.0576444444444455</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
@@ -46444,7 +46450,7 @@
         <v>4.337422222222223</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
@@ -46461,7 +46467,7 @@
         <v>5.0838888888888878</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>16</v>
       </c>
@@ -46478,7 +46484,7 @@
         <v>4.9794000000000009</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
@@ -46495,7 +46501,7 @@
         <v>5.058422222222223</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>20</v>
       </c>
@@ -46512,7 +46518,7 @@
         <v>5.0893333333333342</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
@@ -46529,7 +46535,7 @@
         <v>5.0880444444444439</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>24</v>
       </c>
@@ -46546,7 +46552,7 @@
         <v>4.8201555555555551</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>26</v>
       </c>
@@ -46563,7 +46569,7 @@
         <v>4.5370222222222214</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>3</v>
       </c>
@@ -46580,7 +46586,7 @@
         <v>4.7765555555555554</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>3</v>
       </c>
@@ -47141,7 +47147,7 @@
         <v>5.0551999999999992</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
         <v>25</v>
       </c>
@@ -47158,7 +47164,7 @@
         <v>3.8309333333333337</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>25</v>
       </c>
@@ -47175,7 +47181,7 @@
         <v>4.5995999999999997</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
         <v>27</v>
       </c>
@@ -47192,7 +47198,7 @@
         <v>4.9930000000000003</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
         <v>27</v>
       </c>
@@ -47209,7 +47215,7 @@
         <v>3.4152222222222219</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
         <v>27</v>
       </c>
@@ -47226,7 +47232,7 @@
         <v>4.0032666666666668</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
         <v>2</v>
       </c>
@@ -47242,8 +47248,11 @@
       <c r="E54" s="8">
         <v>4.972488888888889</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F54">
+        <v>4.9383777777777791</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
         <v>2</v>
       </c>
@@ -47259,8 +47268,11 @@
       <c r="E55" s="8">
         <v>3.6407555555555553</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F55">
+        <v>3.6066444444444454</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
         <v>2</v>
       </c>
@@ -47276,8 +47288,11 @@
       <c r="E56" s="8">
         <v>3.7489777777777777</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F56">
+        <v>3.7148666666666679</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
         <v>4</v>
       </c>
@@ -47293,8 +47308,11 @@
       <c r="E57" s="8">
         <v>5.0205111111111105</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F57">
+        <v>4.6451555555555544</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
         <v>4</v>
       </c>
@@ -47310,8 +47328,11 @@
       <c r="E58" s="8">
         <v>3.4370222222222226</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F58">
+        <v>3.0616666666666665</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
         <v>4</v>
       </c>
@@ -47327,8 +47348,11 @@
       <c r="E59" s="8">
         <v>4.2691777777777773</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F59">
+        <v>3.8938222222222212</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
         <v>6</v>
       </c>
@@ -47344,8 +47368,11 @@
       <c r="E60" s="8">
         <v>4.9493777777777783</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F60">
+        <v>4.7206222222222216</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
         <v>6</v>
       </c>
@@ -47361,8 +47388,11 @@
       <c r="E61" s="8">
         <v>2.9934000000000007</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F61">
+        <v>2.764644444444444</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
         <v>6</v>
       </c>
@@ -47378,8 +47408,11 @@
       <c r="E62" s="8">
         <v>3.7731111111111106</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F62">
+        <v>3.5443555555555539</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
         <v>8</v>
       </c>
@@ -47395,8 +47428,11 @@
       <c r="E63" s="8">
         <v>5.0744666666666678</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F63">
+        <v>5.516466666666668</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
         <v>8</v>
       </c>
@@ -47412,8 +47448,11 @@
       <c r="E64" s="8">
         <v>2.5238444444444434</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F64">
+        <v>2.9658444444444436</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>8</v>
       </c>
@@ -47429,8 +47468,11 @@
       <c r="E65" s="8">
         <v>3.0262888888888897</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F65">
+        <v>3.4682888888888899</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
         <v>10</v>
       </c>
@@ -47446,8 +47488,11 @@
       <c r="E66" s="8">
         <v>5.007822222222222</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F66">
+        <v>4.9501777777777765</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
         <v>10</v>
       </c>
@@ -47463,8 +47508,11 @@
       <c r="E67" s="8">
         <v>2.3152888888888898</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F67">
+        <v>2.2576444444444443</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
         <v>10</v>
       </c>
@@ -47480,8 +47528,11 @@
       <c r="E68" s="8">
         <v>2.634155555555556</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F68">
+        <v>2.5765111111111105</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
         <v>12</v>
       </c>
@@ -47497,8 +47548,11 @@
       <c r="E69" s="8">
         <v>4.4893333333333336</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F69">
+        <v>5.1519111111111107</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
         <v>12</v>
       </c>
@@ -47514,8 +47568,11 @@
       <c r="E70" s="8">
         <v>3.3160444444444437</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F70">
+        <v>3.9786222222222207</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
         <v>12</v>
       </c>
@@ -47531,8 +47588,11 @@
       <c r="E71" s="8">
         <v>3.8448444444444445</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F71">
+        <v>4.5074222222222211</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
         <v>14</v>
       </c>
@@ -47548,8 +47608,11 @@
       <c r="E72" s="8">
         <v>5.0587777777777774</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F72">
+        <v>4.9748888888888896</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="s">
         <v>14</v>
       </c>
@@ -47565,8 +47628,11 @@
       <c r="E73" s="8">
         <v>2.8551111111111114</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F73">
+        <v>2.7712222222222236</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
         <v>14</v>
       </c>
@@ -47582,8 +47648,11 @@
       <c r="E74" s="8">
         <v>3.6996444444444441</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F74">
+        <v>3.6157555555555563</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
         <v>16</v>
       </c>
@@ -47599,8 +47668,11 @@
       <c r="E75" s="8">
         <v>5.0275555555555567</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F75">
+        <v>5.0481555555555557</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
         <v>16</v>
       </c>
@@ -47616,8 +47688,11 @@
       <c r="E76" s="8">
         <v>3.0592888888888883</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F76">
+        <v>3.0798888888888873</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="3" t="s">
         <v>16</v>
       </c>
@@ -47633,8 +47708,11 @@
       <c r="E77" s="8">
         <v>3.9506444444444448</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F77">
+        <v>3.9712444444444439</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="3" t="s">
         <v>18</v>
       </c>
@@ -47650,8 +47728,11 @@
       <c r="E78" s="8">
         <v>5.0608666666666675</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F78">
+        <v>5.0024444444444445</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="3" t="s">
         <v>18</v>
       </c>
@@ -47667,8 +47748,11 @@
       <c r="E79" s="8">
         <v>2.5296222222222227</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F79">
+        <v>2.4711999999999996</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" s="3" t="s">
         <v>18</v>
       </c>
@@ -47684,8 +47768,11 @@
       <c r="E80" s="8">
         <v>3.4427555555555562</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F80">
+        <v>3.3843333333333332</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" s="3" t="s">
         <v>20</v>
       </c>
@@ -47701,8 +47788,11 @@
       <c r="E81" s="8">
         <v>4.897955555555555</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F81">
+        <v>4.8086222222222208</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="3" t="s">
         <v>20</v>
       </c>
@@ -47718,8 +47808,11 @@
       <c r="E82" s="8">
         <v>2.4876444444444452</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F82">
+        <v>2.3983111111111111</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" s="3" t="s">
         <v>20</v>
       </c>
@@ -47735,8 +47828,11 @@
       <c r="E83" s="8">
         <v>2.9646444444444437</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F83">
+        <v>2.8753111111111096</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" s="3" t="s">
         <v>22</v>
       </c>
@@ -47752,8 +47848,11 @@
       <c r="E84" s="8">
         <v>4.9810222222222214</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F84">
+        <v>4.8929777777777774</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" s="3" t="s">
         <v>22</v>
       </c>
@@ -47769,8 +47868,11 @@
       <c r="E85" s="8">
         <v>3.5219111111111112</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F85">
+        <v>3.4338666666666673</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
         <v>22</v>
       </c>
@@ -47786,8 +47888,11 @@
       <c r="E86" s="8">
         <v>4.288044444444445</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F86">
+        <v>4.2000000000000011</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="s">
         <v>24</v>
       </c>
@@ -47803,8 +47908,11 @@
       <c r="E87" s="8">
         <v>4.9855999999999998</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F87">
+        <v>5.1654444444444447</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" s="3" t="s">
         <v>24</v>
       </c>
@@ -47820,8 +47928,11 @@
       <c r="E88" s="8">
         <v>3.0415555555555556</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F88">
+        <v>3.2214000000000005</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
         <v>24</v>
       </c>
@@ -47837,8 +47948,11 @@
       <c r="E89" s="8">
         <v>3.9174222222222226</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F89">
+        <v>4.0972666666666679</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="s">
         <v>26</v>
       </c>
@@ -47854,8 +47968,11 @@
       <c r="E90" s="8">
         <v>4.9394666666666662</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F90">
+        <v>5.4024444444444448</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" s="3" t="s">
         <v>26</v>
       </c>
@@ -47871,8 +47988,11 @@
       <c r="E91" s="8">
         <v>3.2345555555555556</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F91">
+        <v>3.6975333333333342</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" s="3" t="s">
         <v>26</v>
       </c>
@@ -47888,8 +48008,11 @@
       <c r="E92" s="8">
         <v>3.6752444444444445</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F92">
+        <v>4.1382222222222236</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" s="3" t="s">
         <v>3</v>
       </c>
@@ -47906,7 +48029,7 @@
         <v>5.0539777777777779</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="s">
         <v>5</v>
       </c>
@@ -47923,7 +48046,7 @@
         <v>4.9769333333333332</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" s="3" t="s">
         <v>7</v>
       </c>
@@ -47940,7 +48063,7 @@
         <v>4.8559777777777784</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" s="3" t="s">
         <v>9</v>
       </c>
@@ -48501,7 +48624,7 @@
         <v>4.4732666666666674</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" s="3" t="s">
         <v>21</v>
       </c>
@@ -48518,7 +48641,7 @@
         <v>4.3938444444444444</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" s="3" t="s">
         <v>21</v>
       </c>
@@ -48535,7 +48658,7 @@
         <v>2.5789777777777774</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" s="3" t="s">
         <v>21</v>
       </c>
@@ -48552,7 +48675,7 @@
         <v>3.877844444444444</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" s="3" t="s">
         <v>23</v>
       </c>
@@ -48569,7 +48692,7 @@
         <v>4.8847777777777779</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" s="3" t="s">
         <v>23</v>
       </c>
@@ -48586,7 +48709,7 @@
         <v>2.8127111111111103</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" s="3" t="s">
         <v>23</v>
       </c>
@@ -48603,7 +48726,7 @@
         <v>3.7045111111111102</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" s="3" t="s">
         <v>25</v>
       </c>
@@ -48620,7 +48743,7 @@
         <v>5.3477777777777771</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" s="3" t="s">
         <v>25</v>
       </c>
@@ -48637,7 +48760,7 @@
         <v>3.9358222222222223</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" s="3" t="s">
         <v>25</v>
       </c>
@@ -48654,7 +48777,7 @@
         <v>4.9591777777777786</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" s="3" t="s">
         <v>27</v>
       </c>
@@ -48671,7 +48794,7 @@
         <v>5.5366888888888877</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" s="3" t="s">
         <v>27</v>
       </c>
@@ -48688,7 +48811,7 @@
         <v>3.7868444444444442</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" s="3" t="s">
         <v>27</v>
       </c>
@@ -48705,7 +48828,7 @@
         <v>4.9341333333333326</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" s="3" t="s">
         <v>2</v>
       </c>
@@ -48721,8 +48844,11 @@
       <c r="E141" s="8">
         <v>4.6538666666666657</v>
       </c>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F141">
+        <v>4.6197555555555558</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" s="3" t="s">
         <v>2</v>
       </c>
@@ -48738,8 +48864,11 @@
       <c r="E142" s="8">
         <v>2.4810222222222222</v>
       </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F142">
+        <v>2.4469111111111124</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" s="3" t="s">
         <v>4</v>
       </c>
@@ -48755,8 +48884,11 @@
       <c r="E143" s="8">
         <v>4.907</v>
       </c>
-    </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F143">
+        <v>4.5316444444444439</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" s="3" t="s">
         <v>4</v>
       </c>
@@ -48772,8 +48904,11 @@
       <c r="E144" s="8">
         <v>2.4436666666666671</v>
       </c>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F144">
+        <v>2.068311111111111</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" s="3" t="s">
         <v>6</v>
       </c>
@@ -48789,8 +48924,11 @@
       <c r="E145" s="8">
         <v>4.81768888888889</v>
       </c>
-    </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F145">
+        <v>4.5889333333333333</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" s="3" t="s">
         <v>6</v>
       </c>
@@ -48806,8 +48944,11 @@
       <c r="E146" s="8">
         <v>2.173688888888889</v>
       </c>
-    </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F146">
+        <v>1.9449333333333323</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" s="3" t="s">
         <v>6</v>
       </c>
@@ -48823,8 +48964,11 @@
       <c r="E147" s="8">
         <v>2.508688888888889</v>
       </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F147">
+        <v>2.2799333333333323</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148" s="3" t="s">
         <v>8</v>
       </c>
@@ -48840,8 +48984,11 @@
       <c r="E148" s="8">
         <v>5.0443999999999987</v>
       </c>
-    </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F148">
+        <v>5.4863999999999988</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" s="3" t="s">
         <v>8</v>
       </c>
@@ -48857,8 +49004,11 @@
       <c r="E149" s="8">
         <v>2.2337111111111101</v>
       </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F149">
+        <v>2.6757111111111103</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" s="3" t="s">
         <v>8</v>
       </c>
@@ -48874,8 +49024,11 @@
       <c r="E150" s="8">
         <v>3.322466666666668</v>
       </c>
-    </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F150">
+        <v>3.7644666666666682</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" s="3" t="s">
         <v>10</v>
       </c>
@@ -48891,8 +49044,11 @@
       <c r="E151" s="8">
         <v>4.9913333333333316</v>
       </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F151">
+        <v>4.9336888888888861</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152" s="3" t="s">
         <v>10</v>
       </c>
@@ -48908,8 +49064,11 @@
       <c r="E152" s="8">
         <v>2.0230222222222221</v>
       </c>
-    </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F152">
+        <v>1.9653777777777766</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" s="3" t="s">
         <v>10</v>
       </c>
@@ -48925,8 +49084,11 @@
       <c r="E153" s="8">
         <v>3.1460888888888885</v>
       </c>
-    </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F153">
+        <v>3.088444444444443</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" s="3" t="s">
         <v>12</v>
       </c>
@@ -48942,8 +49104,11 @@
       <c r="E154" s="8">
         <v>4.919777777777778</v>
       </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F154">
+        <v>5.5823555555555551</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A155" s="3" t="s">
         <v>12</v>
       </c>
@@ -48959,8 +49124,11 @@
       <c r="E155" s="8">
         <v>2.4357999999999995</v>
       </c>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F155">
+        <v>3.0983777777777766</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A156" s="3" t="s">
         <v>12</v>
       </c>
@@ -48976,8 +49144,11 @@
       <c r="E156" s="8">
         <v>3.8761333333333341</v>
       </c>
-    </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F156">
+        <v>4.5387111111111107</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A157" s="3" t="s">
         <v>14</v>
       </c>
@@ -48993,8 +49164,11 @@
       <c r="E157" s="8">
         <v>4.969955555555555</v>
       </c>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F157">
+        <v>4.8860666666666672</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A158" s="3" t="s">
         <v>14</v>
       </c>
@@ -49010,8 +49184,11 @@
       <c r="E158" s="8">
         <v>2.1526222222222229</v>
       </c>
-    </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F158">
+        <v>2.0687333333333351</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A159" s="3" t="s">
         <v>14</v>
       </c>
@@ -49027,8 +49204,11 @@
       <c r="E159" s="8">
         <v>2.9761111111111109</v>
       </c>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F159">
+        <v>2.8922222222222231</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A160" s="3" t="s">
         <v>16</v>
       </c>
@@ -49044,8 +49224,11 @@
       <c r="E160" s="8">
         <v>5.0185111111111098</v>
       </c>
-    </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F160">
+        <v>5.0391111111111089</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161" s="3" t="s">
         <v>16</v>
       </c>
@@ -49061,8 +49244,11 @@
       <c r="E161" s="8">
         <v>1.9132000000000002</v>
       </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F161">
+        <v>1.9337999999999993</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162" s="3" t="s">
         <v>16</v>
       </c>
@@ -49078,8 +49264,11 @@
       <c r="E162" s="8">
         <v>3.1115333333333339</v>
       </c>
-    </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F162">
+        <v>3.132133333333333</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163" s="3" t="s">
         <v>18</v>
       </c>
@@ -49095,8 +49284,11 @@
       <c r="E163" s="8">
         <v>4.8448222222222226</v>
       </c>
-    </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F163">
+        <v>4.7863999999999995</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164" s="3" t="s">
         <v>18</v>
       </c>
@@ -49112,8 +49304,11 @@
       <c r="E164" s="8">
         <v>2.079022222222223</v>
       </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F164">
+        <v>2.0206</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165" s="3" t="s">
         <v>18</v>
       </c>
@@ -49129,8 +49324,11 @@
       <c r="E165" s="8">
         <v>3.2646222222222221</v>
       </c>
-    </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F165">
+        <v>3.2061999999999991</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A166" s="3" t="s">
         <v>20</v>
       </c>
@@ -49146,8 +49344,11 @@
       <c r="E166" s="8">
         <v>4.9629555555555553</v>
       </c>
-    </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F166">
+        <v>4.8736222222222212</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A167" s="3" t="s">
         <v>20</v>
       </c>
@@ -49163,8 +49364,11 @@
       <c r="E167" s="8">
         <v>1.9230222222222224</v>
       </c>
-    </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F167">
+        <v>1.8336888888888883</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A168" s="3" t="s">
         <v>20</v>
       </c>
@@ -49180,8 +49384,11 @@
       <c r="E168" s="8">
         <v>2.7789777777777775</v>
       </c>
-    </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F168">
+        <v>2.6896444444444434</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A169" s="3" t="s">
         <v>22</v>
       </c>
@@ -49197,8 +49404,11 @@
       <c r="E169" s="8">
         <v>4.901644444444444</v>
       </c>
-    </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F169">
+        <v>4.8136000000000001</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A170" s="3" t="s">
         <v>22</v>
       </c>
@@ -49214,8 +49424,11 @@
       <c r="E170" s="8">
         <v>2.2358222222222222</v>
       </c>
-    </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F170">
+        <v>2.1477777777777782</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A171" s="3" t="s">
         <v>24</v>
       </c>
@@ -49231,8 +49444,11 @@
       <c r="E171" s="8">
         <v>5.1139777777777784</v>
       </c>
-    </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F171">
+        <v>5.2938222222222233</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A172" s="3" t="s">
         <v>24</v>
       </c>
@@ -49248,8 +49464,11 @@
       <c r="E172" s="8">
         <v>2.6180666666666665</v>
       </c>
-    </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F172">
+        <v>2.7979111111111115</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A173" s="3" t="s">
         <v>24</v>
       </c>
@@ -49265,8 +49484,11 @@
       <c r="E173" s="8">
         <v>3.8469111111111109</v>
       </c>
-    </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F173">
+        <v>4.0267555555555559</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A174" s="3" t="s">
         <v>26</v>
       </c>
@@ -49282,8 +49504,11 @@
       <c r="E174" s="8">
         <v>5.1320888888888891</v>
       </c>
-    </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F174">
+        <v>5.5950666666666677</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A175" s="3" t="s">
         <v>26</v>
       </c>
@@ -49299,8 +49524,11 @@
       <c r="E175" s="8">
         <v>2.8756666666666666</v>
       </c>
-    </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F175">
+        <v>3.3386444444444452</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A176" s="3" t="s">
         <v>26</v>
       </c>
@@ -49316,8 +49544,11 @@
       <c r="E176" s="8">
         <v>4.9189999999999987</v>
       </c>
-    </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F176">
+        <v>5.3819777777777773</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A177" s="3" t="s">
         <v>2</v>
       </c>
@@ -49333,8 +49564,11 @@
       <c r="E177" s="8">
         <v>5.0012222222222222</v>
       </c>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F177">
+        <v>4.9671111111111124</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A178" s="3" t="s">
         <v>2</v>
       </c>
@@ -49350,8 +49584,11 @@
       <c r="E178" s="8">
         <v>3.7263111111111114</v>
       </c>
-    </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F178">
+        <v>3.6922000000000015</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A179" s="3" t="s">
         <v>2</v>
       </c>
@@ -49367,8 +49604,11 @@
       <c r="E179" s="8">
         <v>4.2139111111111118</v>
       </c>
-    </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F179">
+        <v>4.179800000000002</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A180" s="3" t="s">
         <v>4</v>
       </c>
@@ -49384,8 +49624,11 @@
       <c r="E180" s="8">
         <v>5.0883555555555553</v>
       </c>
-    </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F180">
+        <v>4.7129999999999992</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A181" s="3" t="s">
         <v>4</v>
       </c>
@@ -49401,8 +49644,11 @@
       <c r="E181" s="8">
         <v>3.5568444444444434</v>
       </c>
-    </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F181">
+        <v>3.1814888888888873</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A182" s="3" t="s">
         <v>4</v>
       </c>
@@ -49418,8 +49664,11 @@
       <c r="E182" s="8">
         <v>3.8699555555555558</v>
       </c>
-    </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F182">
+        <v>3.4945999999999997</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A183" s="3" t="s">
         <v>6</v>
       </c>
@@ -49435,8 +49684,11 @@
       <c r="E183" s="8">
         <v>4.8740444444444435</v>
       </c>
-    </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F183">
+        <v>4.6452888888888868</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A184" s="3" t="s">
         <v>6</v>
       </c>
@@ -49452,8 +49704,11 @@
       <c r="E184" s="8">
         <v>3.046044444444445</v>
       </c>
-    </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F184">
+        <v>2.8172888888888883</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A185" s="3" t="s">
         <v>6</v>
       </c>
@@ -49469,8 +49724,11 @@
       <c r="E185" s="8">
         <v>4.1036888888888896</v>
       </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F185">
+        <v>3.8749333333333329</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A186" s="3" t="s">
         <v>8</v>
       </c>
@@ -49486,8 +49744,11 @@
       <c r="E186" s="8">
         <v>4.4168888888888898</v>
       </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F186">
+        <v>4.8588888888888899</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A187" s="3" t="s">
         <v>8</v>
       </c>
@@ -49503,8 +49764,11 @@
       <c r="E187" s="8">
         <v>2.5612666666666657</v>
       </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F187">
+        <v>3.0032666666666659</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A188" s="3" t="s">
         <v>8</v>
       </c>
@@ -49520,8 +49784,11 @@
       <c r="E188" s="8">
         <v>3.2773777777777768</v>
       </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F188">
+        <v>3.719377777777777</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A189" s="3" t="s">
         <v>10</v>
       </c>
@@ -49537,8 +49804,11 @@
       <c r="E189" s="8">
         <v>4.9098444444444436</v>
       </c>
-    </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F189">
+        <v>4.8521999999999981</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A190" s="3" t="s">
         <v>10</v>
       </c>
@@ -49554,8 +49824,11 @@
       <c r="E190" s="8">
         <v>2.235844444444445</v>
       </c>
-    </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F190">
+        <v>2.1781999999999995</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A191" s="3" t="s">
         <v>10</v>
       </c>
@@ -49571,8 +49844,11 @@
       <c r="E191" s="8">
         <v>3.0641555555555562</v>
       </c>
-    </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F191">
+        <v>3.0065111111111107</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A192" s="3" t="s">
         <v>12</v>
       </c>
@@ -49588,8 +49864,11 @@
       <c r="E192" s="8">
         <v>4.8868666666666662</v>
       </c>
-    </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F192">
+        <v>5.5494444444444433</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A193" s="3" t="s">
         <v>12</v>
       </c>
@@ -49605,8 +49884,11 @@
       <c r="E193" s="8">
         <v>3.0173333333333332</v>
       </c>
-    </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F193">
+        <v>3.6799111111111102</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A194" s="3" t="s">
         <v>12</v>
       </c>
@@ -49622,8 +49904,11 @@
       <c r="E194" s="8">
         <v>3.5226444444444436</v>
       </c>
-    </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F194">
+        <v>4.1852222222222206</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A195" s="3" t="s">
         <v>14</v>
       </c>
@@ -49639,8 +49924,11 @@
       <c r="E195" s="8">
         <v>4.7217777777777759</v>
       </c>
-    </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F195">
+        <v>4.6378888888888881</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A196" s="3" t="s">
         <v>14</v>
       </c>
@@ -49656,8 +49944,11 @@
       <c r="E196" s="8">
         <v>2.9050000000000002</v>
       </c>
-    </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F196">
+        <v>2.8211111111111125</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A197" s="3" t="s">
         <v>14</v>
       </c>
@@ -49673,8 +49964,11 @@
       <c r="E197" s="8">
         <v>3.7345333333333337</v>
       </c>
-    </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F197">
+        <v>3.6506444444444459</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A198" s="3" t="s">
         <v>16</v>
       </c>
@@ -49690,8 +49984,11 @@
       <c r="E198" s="8">
         <v>5.0518666666666663</v>
       </c>
-    </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F198">
+        <v>5.0724666666666653</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A199" s="3" t="s">
         <v>16</v>
       </c>
@@ -49707,8 +50004,11 @@
       <c r="E199" s="8">
         <v>3.0963555555555562</v>
       </c>
-    </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F199">
+        <v>3.1169555555555553</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A200" s="3" t="s">
         <v>16</v>
       </c>
@@ -49724,8 +50024,11 @@
       <c r="E200" s="8">
         <v>4.4016222222222225</v>
       </c>
-    </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F200">
+        <v>4.4222222222222216</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A201" s="3" t="s">
         <v>18</v>
       </c>
@@ -49741,8 +50044,11 @@
       <c r="E201" s="8">
         <v>4.9106888888888882</v>
       </c>
-    </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F201">
+        <v>4.8522666666666652</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A202" s="3" t="s">
         <v>18</v>
       </c>
@@ -49758,8 +50064,11 @@
       <c r="E202" s="8">
         <v>2.6871777777777783</v>
       </c>
-    </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F202">
+        <v>2.6287555555555553</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A203" s="3" t="s">
         <v>18</v>
       </c>
@@ -49775,8 +50084,11 @@
       <c r="E203" s="8">
         <v>3.0276000000000001</v>
       </c>
-    </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F203">
+        <v>2.969177777777777</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A204" s="3" t="s">
         <v>20</v>
       </c>
@@ -49792,8 +50104,11 @@
       <c r="E204" s="8">
         <v>5.0501777777777779</v>
       </c>
-    </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F204">
+        <v>4.9608444444444437</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A205" s="3" t="s">
         <v>20</v>
       </c>
@@ -49809,8 +50124,11 @@
       <c r="E205" s="8">
         <v>2.529177777777778</v>
       </c>
-    </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F205">
+        <v>2.4398444444444438</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A206" s="3" t="s">
         <v>20</v>
       </c>
@@ -49826,8 +50144,11 @@
       <c r="E206" s="8">
         <v>3.1217777777777767</v>
       </c>
-    </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F206">
+        <v>3.0324444444444425</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A207" s="3" t="s">
         <v>22</v>
       </c>
@@ -49843,8 +50164,11 @@
       <c r="E207" s="8">
         <v>5.0218222222222231</v>
       </c>
-    </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F207">
+        <v>4.9337777777777791</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A208" s="3" t="s">
         <v>22</v>
       </c>
@@ -49860,8 +50184,11 @@
       <c r="E208" s="8">
         <v>2.9192666666666671</v>
       </c>
-    </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F208">
+        <v>2.8312222222222232</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A209" s="3" t="s">
         <v>22</v>
       </c>
@@ -49877,8 +50204,11 @@
       <c r="E209" s="8">
         <v>3.4032888888888895</v>
       </c>
-    </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F209">
+        <v>3.3152444444444455</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A210" s="3" t="s">
         <v>24</v>
       </c>
@@ -49894,8 +50224,11 @@
       <c r="E210" s="8">
         <v>4.9548000000000005</v>
       </c>
-    </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F210">
+        <v>5.1346444444444455</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A211" s="3" t="s">
         <v>24</v>
       </c>
@@ -49911,8 +50244,11 @@
       <c r="E211" s="8">
         <v>3.2979111111111115</v>
       </c>
-    </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F211">
+        <v>3.4777555555555564</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A212" s="3" t="s">
         <v>24</v>
       </c>
@@ -49928,8 +50264,11 @@
       <c r="E212" s="8">
         <v>3.6551333333333336</v>
       </c>
-    </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F212">
+        <v>3.8349777777777785</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A213" s="3" t="s">
         <v>26</v>
       </c>
@@ -49945,8 +50284,11 @@
       <c r="E213" s="8">
         <v>4.8502222222222242</v>
       </c>
-    </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F213">
+        <v>5.3132000000000028</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A214" s="3" t="s">
         <v>26</v>
       </c>
@@ -49962,8 +50304,11 @@
       <c r="E214" s="8">
         <v>2.9782222222222221</v>
       </c>
-    </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F214">
+        <v>3.4412000000000007</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A215" s="3" t="s">
         <v>26</v>
       </c>
@@ -49979,8 +50324,11 @@
       <c r="E215" s="8">
         <v>3.5008000000000008</v>
       </c>
-    </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F215">
+        <v>3.9637777777777794</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A216" s="3" t="s">
         <v>3</v>
       </c>
@@ -49997,7 +50345,7 @@
         <v>4.4217111111111116</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A217" s="3" t="s">
         <v>3</v>
       </c>
@@ -50014,7 +50362,7 @@
         <v>3.4345999999999997</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A218" s="3" t="s">
         <v>3</v>
       </c>
@@ -50031,7 +50379,7 @@
         <v>3.886822222222222</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A219" s="3" t="s">
         <v>5</v>
       </c>
@@ -50048,7 +50396,7 @@
         <v>4.232111111111112</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A220" s="3" t="s">
         <v>5</v>
       </c>
@@ -50065,7 +50413,7 @@
         <v>3.5197111111111123</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A221" s="3" t="s">
         <v>5</v>
       </c>
@@ -50082,7 +50430,7 @@
         <v>4.3564000000000007</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A222" s="3" t="s">
         <v>7</v>
       </c>
@@ -50099,7 +50447,7 @@
         <v>4.7214444444444457</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A223" s="3" t="s">
         <v>7</v>
       </c>
@@ -50116,7 +50464,7 @@
         <v>2.9856222222222231</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A224" s="3" t="s">
         <v>7</v>
       </c>

</xml_diff>